<commit_message>
Leads: 2026-10-16 16:27 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://www.gcsheatingcooling.com/</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>office@gcsguys.com</t>
@@ -554,6 +553,66 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Melo Air</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>meloair.net</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.meloair.net/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Verified Customer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>meloair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(813) 451-9438</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>80</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tampa FL</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-16 16:33 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -618,6 +618,126 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A Plus Plumbing and Drains</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>aplusplumbinganddrains.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://aplusplumbinganddrains.com/plumber-thornton-co/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Plus Plumbing</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>aplusplumbinganddrains@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(720) 692-9926</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>plumber Thornton CO</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Plumber in Thornton, CO | Emergency, Drains &amp; Water Heaters</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>plumberthorntonco.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://plumberthorntonco.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Thornton Checklist</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@plumberthorntonco.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(720) 856-5811</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>plumber Thornton CO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-16 16:36 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,186 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A&amp;M Heating and Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>amheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.amheatingandairconditioning.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Air Conditioning</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@amheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(916) 747-5654</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>heating and cooling company Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AC Repair &amp; Installation in New Braunfels, TX - Ductman AC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ductmanac.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://ductmanac.com/ac-repair-and-installation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>New Braunfels</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>jantzen@ductmanac.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(830) 261-4178</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>AC installation New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Climate Express Home Services - New Braunfels Cooling &amp; Heating Services</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>climateexpressair.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.climateexpressair.com/air-conditioner/installation</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>New Braunfels</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>admin@climateexpressair.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>830-302-7401</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>AC installation New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-16 16:37 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,62 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Hi-Tech Plumbing Services inc.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hitechplumbingservicesinc.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://hitechplumbingservicesinc.com/services/emergency-plumber-los-angeles/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>hi_techplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>818-941-6741</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>emergency plumber Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-16 16:45 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -939,7 +939,6 @@
           <t>https://hitechplumbingservicesinc.com/services/emergency-plumber-los-angeles/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>hi_techplumbing@yahoo.com</t>
@@ -969,6 +968,126 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Patriot HVAC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>patriothvac.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://patriothvac.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Some Patriots</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@patriothvac.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>435-288-0408</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>HVAC contractor St George UT</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HVAC Services in Saint George UT | Prompt Local Dispatch | HVAC Saint George</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>hvacsaintgeorge.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>http://hvacsaintgeorge.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Saint George</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>dispatch@hvacsaintgeorge.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(435) 348-8603</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>78</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>HVAC contractor St George UT</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-16 16:48 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1093,6 +1093,66 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Civive Air Services</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>civiveairservices.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://civiveairservices.com/heating-repair</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Scott Berry</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>scott@civiveairservices.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>417-855-4141</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Springfield MO</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>furnace repair Springfield MO</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-16 22:43 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1153,6 +1153,182 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Phoenix Roofing Systems</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>phoenixroofingsystems.net</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://phoenixroofingsystems.net/roofing-in-athens-ga/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Broad Street</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>inquiry@phoenixroofingsystems.net</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>706-636-7663</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Athens GA</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>residential roofing company Athens GA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HVAC Topeka KS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>hvactopekaks.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://hvactopekaks.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Electrical Code</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>dispatch@hvactopekaks.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(785) 219-8054</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Topeka KS</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>heating and cooling company Topeka KS</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation &amp; Service in Ann Arbor</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>fadisheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://fadisheatingcooling.com/locations/ann-arbor-mi/heat-pump-installation-service</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@fadisheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(866) 790-0071</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>heat pump installation Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-16 22:48 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1294,7 +1294,6 @@
           <t>https://fadisheatingcooling.com/locations/ann-arbor-mi/heat-pump-installation-service</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@fadisheatingcooling.com</t>
@@ -1324,6 +1323,66 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ProAir Conditioning</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>proairconditioning.site</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>http://proairconditioning.site/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Plant City</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ethan@proairconditioning.site</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(214) 948-3345</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>88</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>HVAC contractor Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-16 22:56 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-16.xlsx
+++ b/output/leads_2026-10-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1388,6 +1388,66 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>JFK Construction</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>jfkconstructionrgv.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://jfkconstructionrgv.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Hurricane Hanna</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>jfkconstruction2014@gmail.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>956-562-5821</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>82</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>roofing contractor McAllen TX</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>